<commit_message>
Refine mappings in CdaADToAddressConceptMap
Updated descriptions and display names for elements in the ConceptMap to provide clearer mappings from CDA AD to FHIR Address. f693f03763f720da16b1f4bb580c8d68699f457e
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaADToAddressConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaADToAddressConceptMap.xlsx
@@ -8,12 +8,14 @@
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Mapping Table 0" r:id="rId4" sheetId="2"/>
+    <sheet name="Mapping Table 1" r:id="rId5" sheetId="3"/>
+    <sheet name="Mapping Table 2" r:id="rId6" sheetId="4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +26,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaAddressToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaADToAddressConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T09:26:13+00:00</t>
+    <t>2026-07-22T09:42:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +86,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Correspondances documentaires des composants AD vers Address.</t>
+    <t>Correspondances documentaires des composants du type CDA AD vers le type FHIR Address et les extensions associées.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -117,67 +119,115 @@
     <t>AD.item.country</t>
   </si>
   <si>
+    <t>Country</t>
+  </si>
+  <si>
     <t>equivalent</t>
   </si>
   <si>
     <t>Address.country</t>
   </si>
   <si>
+    <t>Country (e.g. can be ISO 3166 2 or 3 letter code)</t>
+  </si>
+  <si>
     <t>AD.item.state</t>
   </si>
   <si>
+    <t>State</t>
+  </si>
+  <si>
     <t>Address.state</t>
   </si>
   <si>
+    <t>Sub-unit of country (abbreviations ok)</t>
+  </si>
+  <si>
     <t>AD.item.county</t>
   </si>
   <si>
+    <t>County</t>
+  </si>
+  <si>
     <t>related-to</t>
   </si>
   <si>
     <t>Address.district</t>
   </si>
   <si>
+    <t>District name (aka county)</t>
+  </si>
+  <si>
     <t>AD.item.city</t>
   </si>
   <si>
+    <t>City</t>
+  </si>
+  <si>
     <t>Address.city</t>
   </si>
   <si>
+    <t>Name of city, town etc.</t>
+  </si>
+  <si>
     <t>AD.item.postalCode</t>
   </si>
   <si>
+    <t>Postal Code</t>
+  </si>
+  <si>
     <t>Address.postalCode</t>
   </si>
   <si>
+    <t>Postal code for area</t>
+  </si>
+  <si>
     <t>AD.item.streetAddressLine</t>
   </si>
   <si>
+    <t>Street Address Line</t>
+  </si>
+  <si>
     <t>Address.line</t>
   </si>
   <si>
+    <t>Street name, number, direction &amp; P.O. Box etc.</t>
+  </si>
+  <si>
+    <t>AD.useablePeriod</t>
+  </si>
+  <si>
+    <t>Useable Period</t>
+  </si>
+  <si>
+    <t>Address.period</t>
+  </si>
+  <si>
+    <t>Time period when address was/is in use</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-streetName|5.3.0</t>
+  </si>
+  <si>
     <t>AD.item.streetName</t>
   </si>
   <si>
-    <t>Address.line.extension[iso21090-ADXP-streetName].valueString</t>
-  </si>
-  <si>
-    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-streetName].valueString</t>
+    <t>Street Name</t>
+  </si>
+  <si>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
+    <t>Value of extension</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-houseNumber|5.3.0</t>
   </si>
   <si>
     <t>AD.item.houseNumber</t>
   </si>
   <si>
-    <t>Address.line.extension[iso21090-ADXP-houseNumber].valueString</t>
-  </si>
-  <si>
-    <t>Address.line.extension[http://hl7.org/fhir/StructureDefinition/iso21090-ADXP-houseNumber].valueString</t>
-  </si>
-  <si>
-    <t>AD.useablePeriod</t>
-  </si>
-  <si>
-    <t>Address.period</t>
+    <t>House Number</t>
   </si>
 </sst>
 </file>
@@ -433,7 +483,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -475,152 +525,240 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="B10" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="C10" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="D10" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="E10" t="s" s="2">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="B11" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="C11" t="s" s="2">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="E11" t="s" s="2">
-        <v>54</v>
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>69</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>